<commit_message>
research: club team-counts across Canada — 419 counted rows from 136 league pages
31 sonnet miners over known RAMP/Kreezee/TeamLinkt league sites (10 leagues
uncountable → skipped, not estimated) + Opus 4.8 spot-check (11 confirmed,
1 refuted: DC Blues 7→11, DCB Red Rush merged per correction). Club Sizes
tabs: Canada-wide in master + per-province workbooks. Directional data for
marketing targeting, evidence line per row.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/research/provinces/SportsHub-Manitoba.xlsx
+++ b/docs/research/provinces/SportsHub-Manitoba.xlsx
@@ -11,12 +11,14 @@
     <sheet name="Leagues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Club-League Map" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Contacts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Club Sizes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs'!$A$1:$P$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leagues'!$A$1:$L$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Club-League Map'!$A$1:$E$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contacts'!$A$1:$F$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Club Sizes'!$A$1:$C$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -557,27 +559,21 @@
           <t>Altona</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>https://altonabasketball.com/</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Community youth basketball; fields tournament teams ($50/team entry incl. association T-shirt and Basketball Manitoba-provided injury insurance)</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>reported</t>
@@ -615,14 +611,11 @@
           <t>Beausejour (Sunrise School Division area, exact town unconfirmed)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>mhovorka@sunrisesd.ca</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Mary-Jo Hovorka — listed contact (role not stated)</t>
@@ -633,13 +626,11 @@
           <t>Boys basketball, ages 14-17 (per directory listing)</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>community program (possibly school-community hybrid — contact uses Sunrise School Division email)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -707,13 +698,11 @@
           <t>Fall Bobcat Basketball Academy for Grades 5-8 (historically K-12); annual summer basketball camps; free annual Holiday Hoops youth camp (Grades 3/4-12) at the Healthy Living Centre</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>university-affiliated youth academy/camps (not school-board varsity)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>verified</t>
@@ -781,13 +770,11 @@
           <t>Girls 14U, 16U, 17U club teams; tryouts at Henry Champ and HLC South</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>university-affiliated youth program</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>reported</t>
@@ -865,7 +852,6 @@
           <t>university-affiliated club program</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>verified</t>
@@ -876,7 +862,6 @@
           <t>http://www.gobobcats.ca/juniorbobcats</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -939,7 +924,6 @@
           <t>university-affiliated youth club/academy</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>verified</t>
@@ -977,7 +961,6 @@
           <t>Brandon</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>204-720-7778</t>
@@ -988,7 +971,6 @@
           <t>treedell33@icloud.com</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Wardell Smith — club contact (PSO registry)</t>
@@ -999,13 +981,11 @@
           <t>Boys team age 13</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>primary</t>
@@ -1016,7 +996,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1039,7 +1018,6 @@
           <t>Brandon</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>204-901-0360</t>
@@ -1117,7 +1095,6 @@
           <t>Dauphin</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>204-572-4484</t>
@@ -1143,13 +1120,11 @@
           <t>Club teams: 14U girls, 15U boys, 18U boys (Dauphin + Grandview); hosted club basketball tournament May 2022 for boys &amp; girls teams ages 14-18 ($350/team, 3-game guarantee)</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>community club (volunteer-run; contacts use Mountain View School Division emails, but operates as a club, not a school team)</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>primary</t>
@@ -1187,7 +1162,6 @@
           <t>Morden</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>204-822-5431</t>
@@ -1203,19 +1177,16 @@
           <t>https://morden.ca/recreation-organizations</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>Municipal youth recreational basketball programming (youth rec basketball; 12+ basketball) offered through City of Morden recreation</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>municipal recreation program (no dedicated club found in Morden)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>reported</t>
@@ -1268,14 +1239,11 @@
           <t>recreation@whereyoubelong.ca</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>Boys club teams born 2010-2013; coach with Los Angeles background; venue Niverville Recreation Centre</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>private academy</t>
@@ -1425,19 +1393,16 @@
           <t>https://nivervillerec.ca/programs/</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>Weekly instructional youth basketball ages 6–9 and 9–14 at the CRRC; hosts Jr. NBA Youth Basketball Camp (ages 5–12)</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>town recreation program (multi-sport org)</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>reported</t>
@@ -1480,14 +1445,11 @@
           <t>Niverville Community Resource &amp; Recreation Centre, Niverville, MB (program venue)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://www.wmba.ca/</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Community youth basketball for boys and girls ages 4-18, delivered in Niverville under the Winnipeg Minor Basketball Association's community programming at the Niverville CRRC</t>
@@ -1545,7 +1507,6 @@
           <t>Niverville area (Eastman/Central region)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>204-998-4462</t>
@@ -1581,7 +1542,6 @@
           <t>community nonprofit / league operator with select teams</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1592,7 +1552,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1615,7 +1574,6 @@
           <t>Portage la Prairie</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>204-870-1071</t>
@@ -1626,7 +1584,6 @@
           <t>centralplainsbasketballclub@gmail.com</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Darin Arnold — club contact (PSO registry)</t>
@@ -1647,7 +1604,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1658,7 +1614,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1681,14 +1636,11 @@
           <t>Selkirk</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>selkirkroyalsbb@outlook.com</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>Blake Hamm — club contact (PSO registry)</t>
@@ -1709,7 +1661,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1720,7 +1671,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1748,7 +1698,6 @@
           <t>Lord Selkirk Regional Comprehensive Secondary School, 221 Mercy Street, Selkirk, MB (program base)</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>selkirkroyalsbb@outlook.com</t>
@@ -1779,7 +1728,6 @@
           <t>community nonprofit (feeder club aligned with Lord Selkirk Regional 'Royals' school program but operated as a Basketball Manitoba member club)</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1817,8 +1765,6 @@
           <t>Southern Manitoba (Winkler/Morden area)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>stephen@bigcountrybasketball.com</t>
@@ -1839,13 +1785,11 @@
           <t>Girls club program ages 12-17 plus basketball-specific training &amp; development for all levels (LTAD-based holistic model)</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>private club/training program</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>reported</t>
@@ -1856,7 +1800,6 @@
           <t>https://www.bigcountrybasketball.com/about</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1879,7 +1822,6 @@
           <t>Steinbach</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>204-998-4462</t>
@@ -1957,7 +1899,6 @@
           <t>Steinbach</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>204-998-4462</t>
@@ -2035,8 +1976,6 @@
           <t>Steinbach</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>jdykerman@hsd.ca</t>
@@ -2109,7 +2048,6 @@
           <t>Steinbach</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>204-370-6507</t>
@@ -2187,7 +2125,6 @@
           <t>The Pas</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>204-620-6110</t>
@@ -2213,13 +2150,11 @@
           <t>Youth basketball association programming for The Pas &amp; area (northern Manitoba)</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>primary</t>
@@ -2257,9 +2192,6 @@
           <t>Thompson</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>https://www.instagram.com/juniorbisons/</t>
@@ -2275,13 +2207,11 @@
           <t>Club basketball program based in Thompson; girls club ages 13-17 listed; Junior Bison Thompson athletes received member pricing at Prairie Elite Academy camps held at Wapanohk Community School (Grades 5-12)</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>reported</t>
@@ -2359,7 +2289,6 @@
           <t>private academy/training + club</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2370,7 +2299,6 @@
           <t>https://btbdhoopsxrelentless.ca/</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2393,8 +2321,6 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>prairieelitebasketballacademy@gmail.com</t>
@@ -2415,13 +2341,11 @@
           <t>Female-focused training academy: development camps for girls Grades 7-12 and players camps for boys &amp; girls ages 11-18 held in Winkler (2018); ran 'Prairie Elite South' club team tryouts in Winkler for girls born 2002+ (2019)</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>private academy</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -2459,8 +2383,6 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>winklerbasketballclub@gmail.com</t>
@@ -2533,8 +2455,6 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>winklerminorbasketball@gmail.com</t>
@@ -2545,7 +2465,6 @@
           <t>https://winklerminorbasketball.weebly.com/</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>Spring house league (begins March) for Winkler &amp; area, boys and girls divisions Grades 3&amp;4, 5&amp;6, 7&amp;8; registration $75; mission: promote basketball skill development in young athletes in the Winkler area</t>
@@ -2603,8 +2522,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>204elite@gmail.com</t>
@@ -2635,7 +2552,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2673,14 +2589,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>ambush.club.basketball@gmail.com</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>Jaira Labelle — club contact (PSO registry)</t>
@@ -2701,7 +2614,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2712,7 +2624,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2735,8 +2646,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>atlasbball@gmail.com</t>
@@ -2767,7 +2676,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2778,7 +2686,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2801,7 +2708,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>431-999-7269</t>
@@ -2837,7 +2743,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2875,14 +2780,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>attacksouthbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Tara Kelly, Erin Sheldon, Ogo Okwumabua — club contacts (PSO registry)</t>
@@ -2945,17 +2847,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>Boys 18U club team; tryouts at Sturgeon Heights Community Centre</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>community club</t>
@@ -2976,7 +2872,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/Club%20Tryouts?updated-max=2024-07-17T00:00:00-05:00&amp;max-results=50</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2999,15 +2894,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>info@chiefsbball.club</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>Indigenous-focused club in partnership with Interlake Reserve Tribal Council (IRTC); boys &amp; girls born 2011-2013 (earlier U12); low-cost $10 tryouts at Université de Saint-Boniface; IRTC Chiefs also field U21 travel teams for Alberta Indigenous Games</t>
@@ -3023,7 +2914,6 @@
           <t>community nonprofit (Indigenous partnership)</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3143,7 +3033,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>204-500-9033</t>
@@ -3221,7 +3110,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>431-334-5169</t>
@@ -3232,7 +3120,6 @@
           <t>delitembb@gmail.com</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Anton Dziuba — club contact (PSO registry)</t>
@@ -3268,7 +3155,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3373,14 +3259,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>downtowndawgs@outlook.com</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>Jordan Fotheringham — club contact (PSO registry)</t>
@@ -3401,7 +3284,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3412,7 +3294,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3435,15 +3316,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>dynastywpg@gmail.com</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>Girls rep teams, born 2009–2012; tryouts at Sport Manitoba (145 Pacific Ave)</t>
@@ -3506,14 +3383,11 @@
           <t>145 Pacific Avenue, Winnipeg, Manitoba R3B 2Z6</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>empireelitehoops@gmail.com</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>Boys teams born 2008–2014, girls born 2010–2012; trains at BATTLE 204 facility; local, national and USA tournaments; tryouts at Sport for Life Centre and YFC Winnipeg</t>
@@ -3529,7 +3403,6 @@
           <t>community club (nonprofit status unverified)</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3622,7 +3495,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3809,8 +3681,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>ignitebasketballwinnipeg@gmail.com</t>
@@ -3883,27 +3753,21 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>junioralliancebasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>Boys born 2008-2014 and girls born 2009 club teams; tryouts at Red River College Polytech South Gym</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>reported</t>
@@ -3914,7 +3778,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/Club%20Tryouts?updated-max=2025-07-02T00:00:00-05:00&amp;max-results=50</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3937,8 +3800,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>juniorbisonboysbasketball@gmail.com</t>
@@ -3949,13 +3810,11 @@
           <t>https://www.juniorbisonboys.ca/</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>Youth basketball club offering programming to boys ages 12-17</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>community club</t>
@@ -4187,7 +4046,6 @@
           <t>https://www.kirkfieldwestwood.com/</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>WMBA founding community centre (1997); WMBA Foundation outdoor courts on site; fields WMBA catchment teams</t>
@@ -4245,8 +4103,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>mkraus.legacyprep@gmail.com</t>
@@ -4339,7 +4195,6 @@
           <t>https://lindenwoodscc.com/</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>WMBA founding community centre (1997); current WMBA indoor court venue; hosts club tryouts (World Class Hoopers, Ignite, Triumph)</t>
@@ -4397,7 +4252,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>204-292-3018</t>
@@ -4433,7 +4287,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>verified</t>
@@ -4471,7 +4324,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>204-292-3018</t>
@@ -4507,7 +4359,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>verified</t>
@@ -4627,27 +4478,21 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>bballmastery@gmail.com</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>Boys &amp; girls club teams born 2009; Instagram @masterybasketball</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
           <t>reported</t>
@@ -4658,7 +4503,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/Club%20Tryouts?updated-max=2023-12-14T00:00:00-06:00&amp;max-results=50</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4681,8 +4525,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>info@northstarbasketball.ca</t>
@@ -4713,7 +4555,6 @@
           <t>private academy operated by nonprofit foundation</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
           <t>verified</t>
@@ -4771,7 +4612,6 @@
           <t>https://oxfordheights.pointstreaksites.com/view/oxfordheights/sports-1/basketball-4</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>Transcona-area catchment for WMBA basketball; outdoor court (built 2014) hosts WMBA x ELEVATE 3x3 summer league</t>
@@ -4829,7 +4669,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>204-294-7931</t>
@@ -4880,7 +4719,6 @@
           <t>https://www.basketballmanitoba.ca/2024/08/pba-winnipeg-announces-2024-25.html</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4985,11 +4823,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>Boys rep (17U entry in fall league); U18 team referenced in coach bios</t>
@@ -5005,7 +4838,6 @@
           <t>community club (unverified structure)</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -5043,7 +4875,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>204-995-1682</t>
@@ -5094,7 +4925,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5117,7 +4947,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>204-891-0144</t>
@@ -5153,7 +4982,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>verified</t>
@@ -5164,7 +4992,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5187,7 +5014,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>204-951-2070</t>
@@ -5198,7 +5024,6 @@
           <t>wpgrisingstarclub@gmail.com</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>Jarred Suyat, Diowe Bacanto, Jerrold Suyat — club contacts (PSO registry)</t>
@@ -5219,7 +5044,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
           <t>verified</t>
@@ -5339,7 +5163,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>204-299-7918</t>
@@ -5350,7 +5173,6 @@
           <t>wgpsummitbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
           <t>Tara Meneer — club contact (PSO registry)</t>
@@ -5371,7 +5193,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
           <t>verified</t>
@@ -5382,7 +5203,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5405,15 +5225,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>jbourcier28@gmail.com</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>Boys rep team (2008 birth year); tryouts at Sturgeon Heights Community Centre</t>
@@ -5429,7 +5245,6 @@
           <t>community club (unverified structure)</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
           <t>reported</t>
@@ -5440,7 +5255,6 @@
           <t>https://www.basketballmanitoba.ca/2025/08/showtime-basketball-club-announces.html</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5483,7 +5297,6 @@
           <t>https://swcc1.ca/basketball/</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>Community basketball; fields catchment teams in WMBA leagues</t>
@@ -5561,7 +5374,6 @@
           <t>https://swcc1.ca/basketball/</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>WMBA catchment basketball ages 7-17 (7-8 co-ed; 9-12 girls / 9-13 boys; 13-17 girls / 14-17 boys) across Richmond and Waverley sites</t>
@@ -5592,7 +5404,6 @@
           <t>https://swcc1.ca/basketball/</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5615,27 +5426,21 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>wpgwildcatsbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>Girls club teams ages 13-17</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
           <t>community club (girls-focused)</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr">
         <is>
           <t>reported</t>
@@ -5646,7 +5451,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/Club%20Tryouts?updated-max=2023-12-14T00:00:00-06:00&amp;max-results=50</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5669,7 +5473,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>204-914-5663</t>
@@ -5720,7 +5523,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/ClubDirectory</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5743,7 +5545,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>204-333-7005</t>
@@ -5754,7 +5555,6 @@
           <t>unitebasketball22@gmail.com</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>Jordan Lopez — club contact (PSO registry)</t>
@@ -5765,13 +5565,11 @@
           <t>Boys &amp; girls rep teams ages 11–12 and 15–16</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr">
         <is>
           <t>primary</t>
@@ -5814,26 +5612,21 @@
           <t>323 - 145 Pacific Avenue, Winnipeg, Manitoba</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>info@pegcityball.ca</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>Boys club teams born 2008-2010 (2024-25 tryout announcement)</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -5871,11 +5664,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>Boys teams 2009–2011 births and 2011 girls team</t>
@@ -5891,7 +5679,6 @@
           <t>community club (unverified structure)</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -6011,7 +5798,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>204-471-1111</t>
@@ -6027,7 +5813,6 @@
           <t>https://visioneliteacademy.org/basketball</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>Multi-city private academy (Calgary HQ; Winnipeg, Edmonton, Fraser Valley): Vision Academy ages 7-11, Premier League ages 12-17 (internal seasonal league), Vision Basketball Club ages 12-18 competitive; 10-week year-round sessions; pay-per-session options</t>
@@ -6085,14 +5870,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>bballwestside@gmail.com</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>Clarence Vigilance, Coach</t>
@@ -6103,13 +5885,11 @@
           <t>Boys club teams born 2013-2014; tryouts at Sport Manitoba (145 Pacific Ave)</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr">
         <is>
           <t>reported</t>
@@ -6167,7 +5947,6 @@
           <t>https://whyteridge.ca/sports/basketball/</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>House-league basketball via WMBA catchment: ages 7-8 co-ed 3v3, 9-12 (+13 boys), 14-17 (+13 girls) 5v5; fees WMBA $179 + CC $80 + $9 Canada Basketball</t>
@@ -6394,7 +6173,6 @@
           <t>Bronx Park Community Centre, 720 Henderson Hwy (home facility)</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>winnipegblizzards@gmail.com</t>
@@ -6467,8 +6245,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>chaoswinnipeg@gmail.com</t>
@@ -6489,7 +6265,6 @@
           <t>Girls competitive club teams (15U-17U, born 2009-2012); summer/winter skills clinics boys 7-11 and girls 6-18; own outdoor practice courts; travels to national tournaments (BBall Nationals 2025)</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>community club (girls-focused)</t>
@@ -6537,15 +6312,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>jq14@shaw.ca</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
           <t>Boys rep team (2010 birth year); tryouts at Sturgeon Heights Community Centre (210 Rita St.)</t>
@@ -6561,7 +6332,6 @@
           <t>community club (unverified structure)</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
         <is>
           <t>reported</t>
@@ -6572,7 +6342,6 @@
           <t>https://www.basketballmanitoba.ca/2025/08/winnipeg-cobras-basketball-club-hosting.html</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6600,7 +6369,6 @@
           <t>Duckworth Centre, University of Winnipeg, Winnipeg, MB</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>al.cox@uwinnipeg.ca</t>
@@ -6631,7 +6399,6 @@
           <t>university-affiliated club program</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr">
         <is>
           <t>verified</t>
@@ -6674,7 +6441,6 @@
           <t>Duckworth Centre, 400 Spence St, Winnipeg</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>jrwesmen@gmail.com</t>
@@ -6705,7 +6471,6 @@
           <t>university-affiliated youth program (girls)</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
           <t>verified</t>
@@ -6798,7 +6563,6 @@
           <t>https://www.wmba.ca/</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6821,27 +6585,21 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>wpgsaints@gmail.com</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
           <t>Boys club team born 2010; tryouts at Valour Community Centre (715 Telfer St N)</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>community club</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr">
         <is>
           <t>reported</t>
@@ -6852,7 +6610,6 @@
           <t>https://www.basketballmanitoba.ca/search/label/Club%20Tryouts?max-results=100</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6915,7 +6672,6 @@
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>verified</t>
@@ -6926,7 +6682,6 @@
           <t>https://www.winnipegteammayhem.com/en/</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6949,8 +6704,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>winnipegwolves@gmail.com</t>
@@ -6971,7 +6724,6 @@
           <t>Operating since 2006; recent seasons girls U15/U18 teams; training programs; tryouts at Université de Saint-Boniface</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>community club</t>
@@ -7019,11 +6771,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
           <t>Boys team (2010 birth year)</t>
@@ -7039,7 +6786,6 @@
           <t>community club (unverified structure)</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr">
         <is>
           <t>uncertain</t>
@@ -7077,8 +6823,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>worldclasshoopers@gmail.com</t>
@@ -7109,7 +6853,6 @@
           <t>community club (nonprofit status unverified)</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr">
         <is>
           <t>verified</t>
@@ -7177,13 +6920,11 @@
           <t>Free boys club basketball ages 13-17 (grades 8-12), Thursdays Sep-Dec: skills, scrimmages, faith-based mentorship; first-year program forming new teams weekly</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>multi-sport/faith-based charity youth org</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr">
         <is>
           <t>verified</t>
@@ -7194,7 +6935,6 @@
           <t>https://yfc.ca/winnipeg/program/club-basketball/</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7247,13 +6987,11 @@
           <t>Free weekly boys basketball (ages 13–17, Grades 8–12), Thursdays Sept–Dec; skills + scrimmages; facility also hosts club tryouts (e.g., Empire)</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>faith-based charity / multi-sport youth org (registered charity #119307619 RR0001)</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr">
         <is>
           <t>primary</t>
@@ -11196,7 +10934,6 @@
           <t>Beausejour (Sunrise School Division area, exact town unconfirmed)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>mhovorka@sunrisesd.ca</t>
@@ -11207,7 +10944,6 @@
           <t>Mary-Jo Hovorka — listed contact (role not stated)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11363,7 +11099,6 @@
           <t>Wardell Smith — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11450,7 +11185,6 @@
           <t>recreation@mymorden.ca</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>https://morden.ca/recreation-organizations</t>
@@ -11478,8 +11212,6 @@
           <t>recreation@whereyoubelong.ca</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11534,7 +11266,6 @@
           <t>recreation@whereyoubelong.ca</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>https://nivervillerec.ca/programs/</t>
@@ -11599,7 +11330,6 @@
           <t>Darin Arnold — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11612,7 +11342,6 @@
           <t>Selkirk</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>selkirkroyalsbb@outlook.com</t>
@@ -11623,7 +11352,6 @@
           <t>Blake Hamm — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11636,7 +11364,6 @@
           <t>Selkirk</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>selkirkroyalsbb@outlook.com</t>
@@ -11664,7 +11391,6 @@
           <t>Southern Manitoba (Winkler/Morden area)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>stephen@bigcountrybasketball.com</t>
@@ -11756,7 +11482,6 @@
           <t>Steinbach</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>jdykerman@hsd.ca</t>
@@ -11848,8 +11573,6 @@
           <t>Thompson</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Kristin Donovan — listed contact for Thompson girls club (ages 13-17) in the NBA/eCrew 'Find a Place to Play' Manitoba directory</t>
@@ -11904,7 +11627,6 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>prairieelitebasketballacademy@gmail.com</t>
@@ -11932,7 +11654,6 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>winklerbasketballclub@gmail.com</t>
@@ -11960,13 +11681,11 @@
           <t>Winkler</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>winklerminorbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>https://winklerminorbasketball.weebly.com/</t>
@@ -11984,7 +11703,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>204elite@gmail.com</t>
@@ -12012,7 +11730,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>ambush.club.basketball@gmail.com</t>
@@ -12023,7 +11740,6 @@
           <t>Jaira Labelle — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12036,7 +11752,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>atlasbball@gmail.com</t>
@@ -12096,7 +11811,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>attacksouthbasketball@gmail.com</t>
@@ -12107,7 +11821,6 @@
           <t>Tara Kelly, Erin Sheldon, Ogo Okwumabua — club contacts (PSO registry)</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12120,14 +11833,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>info@chiefsbball.club</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12219,7 +11929,6 @@
           <t>Anton Dziuba — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -12264,7 +11973,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>downtowndawgs@outlook.com</t>
@@ -12275,7 +11983,6 @@
           <t>Jordan Fotheringham — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12288,14 +11995,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>dynastywpg@gmail.com</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -12308,14 +12012,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>empireelitehoops@gmail.com</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -12424,7 +12125,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>ignitebasketballwinnipeg@gmail.com</t>
@@ -12452,14 +12152,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>junioralliancebasketball@gmail.com</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -12472,13 +12169,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>juniorbisonboysbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>https://www.juniorbisonboys.ca/</t>
@@ -12570,7 +12265,6 @@
           <t>office@kwcc.net</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>https://www.kirkfieldwestwood.com/</t>
@@ -12588,7 +12282,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>mkraus.legacyprep@gmail.com</t>
@@ -12626,7 +12319,6 @@
           <t>manager@lindenwoodscc.com</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>https://lindenwoodscc.com/</t>
@@ -12740,14 +12432,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>bballmastery@gmail.com</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -12760,7 +12449,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>info@northstarbasketball.ca</t>
@@ -12798,7 +12486,6 @@
           <t>oxfordheights@shaw.ca</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>https://oxfordheights.pointstreaksites.com/view/oxfordheights/sports-1/basketball-4</t>
@@ -12959,7 +12646,6 @@
           <t>Jarred Suyat, Diowe Bacanto, Jerrold Suyat — club contacts (PSO registry)</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -13019,7 +12705,6 @@
           <t>Tara Meneer — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -13032,14 +12717,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>jbourcier28@gmail.com</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -13062,7 +12744,6 @@
           <t>basketball@swcc1.ca</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>https://swcc1.ca/basketball/</t>
@@ -13090,7 +12771,6 @@
           <t>booking@swcc1.ca</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>https://swcc1.ca/basketball/</t>
@@ -13108,14 +12788,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>wpgwildcatsbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -13175,7 +12852,6 @@
           <t>Jordan Lopez — club contact (PSO registry)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -13188,14 +12864,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>info@pegcityball.ca</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -13250,7 +12923,6 @@
           <t>hello@visioneliteacademy.org</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>https://visioneliteacademy.org/basketball</t>
@@ -13268,7 +12940,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>bballwestside@gmail.com</t>
@@ -13279,7 +12950,6 @@
           <t>Clarence Vigilance, Coach</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13302,7 +12972,6 @@
           <t>Office@whyteridge.ca</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>https://whyteridge.ca/sports/basketball/</t>
@@ -13384,7 +13053,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
           <t>winnipegblizzards@gmail.com</t>
@@ -13412,7 +13080,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>chaoswinnipeg@gmail.com</t>
@@ -13440,14 +13107,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>jq14@shaw.ca</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13460,7 +13124,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>al.cox@uwinnipeg.ca</t>
@@ -13488,7 +13151,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>jrwesmen@gmail.com</t>
@@ -13548,14 +13210,11 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>wpgsaints@gmail.com</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13600,7 +13259,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>winnipegwolves@gmail.com</t>
@@ -13628,7 +13286,6 @@
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>worldclasshoopers@gmail.com</t>
@@ -13713,4 +13370,1091 @@
   <autoFilter ref="A1:F90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Teams counted (directional)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Breakdown (league=teams)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LWCC</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tyndall Park</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Attack Academy</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Southdale</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SWCC (South Winnipeg)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Relentless</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OHCC (Oxford Heights)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Empire</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dakota</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Garden City</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Evolve</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Junior Bisons</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KWCC</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NK</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Whyte Ridge</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Central Plains</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Earl Grey</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rising Star</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Up Next</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>World Class</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Corydon</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Red River</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>East St Paul</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Maples</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RPCC</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Selkirk</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Chiefs</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Crossover</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>REFRESH</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Triumph</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Pythons</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LaSalle</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Riverview</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Girls Got Game</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NGCC</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Brokenhead Ballers</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Greendell</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Steinbach (Jr. Pilots)</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Winakwa</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>WMBA Fall/Winter Community Centre Leag=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Ignite</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Westside</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DElite</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Downtown Dawgs</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Junior Legacy</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Attack South</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Dynasty</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Jr. Bobcats</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Peg City Club Basketball League (CBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Dunk Dynasty</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Raptors</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Splash Bros</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Bubble Bees</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Thrashers</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Bucket Squad</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Terror Squad</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Aura</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Dark Knights</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Golden Snipers</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Hoop Kings</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>HWE</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Splashers</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Strive Elite</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Bam</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Chuzz Elite</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Splash Zone</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>The Rec</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Prairie Basketball League (PBL)=1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C71"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>